<commit_message>
Address code review findings and finalize BI reporting system
</commit_message>
<xml_diff>
--- a/reports/kpi_report.xlsx
+++ b/reports/kpi_report.xlsx
@@ -19,10 +19,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'KPI Summary'!$A$3:$C$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Monthly Revenue'!$A$3:$B$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Monthly Revenue'!$A$3:$B$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Quarterly Revenue'!$A$3:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Product Performance'!$A$3:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Regional Performance'!$A$3:$D$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Product Performance'!$A$3:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Regional Performance'!$A$3:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sales Performance'!$A$3:$B$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Segment Performance'!$A$3:$N$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Revenue Forecast'!$A$3:$D$3</definedName>
@@ -59,7 +59,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +84,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -149,10 +154,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,7 +573,7 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>3030515.2</v>
+        <v>46395.15</v>
       </c>
     </row>
     <row r="5">
@@ -580,7 +588,7 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>3408.9</v>
+        <v>1159.88</v>
       </c>
     </row>
     <row r="6">
@@ -595,7 +603,7 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>889</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -627,7 +635,7 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>144684.09</v>
+        <v>2962.83</v>
       </c>
     </row>
     <row r="9">
@@ -659,7 +667,7 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>186283.31</v>
+        <v>6283.7</v>
       </c>
     </row>
     <row r="11">
@@ -674,7 +682,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>-22.33</v>
+        <v>-52.85</v>
       </c>
     </row>
     <row r="12">
@@ -689,7 +697,7 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>889</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13">
@@ -704,7 +712,7 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>291</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -719,7 +727,7 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>320</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -734,7 +742,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>75.34</v>
+        <v>68.97</v>
       </c>
     </row>
     <row r="16">
@@ -749,7 +757,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>21.33</v>
+        <v>18.31</v>
       </c>
     </row>
     <row r="17">
@@ -765,7 +773,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>AM_5</t>
+          <t>AM_1</t>
         </is>
       </c>
     </row>
@@ -781,7 +789,7 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>678845.98</v>
+        <v>14930.24</v>
       </c>
     </row>
     <row r="19">
@@ -797,7 +805,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>CRM Enterprise</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
@@ -831,7 +839,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>→ Stable</t>
+          <t>↑ Growing</t>
         </is>
       </c>
     </row>
@@ -847,7 +855,7 @@
         </is>
       </c>
       <c r="C22" s="8" t="n">
-        <v>285.59</v>
+        <v>52.49</v>
       </c>
     </row>
     <row r="23">
@@ -862,7 +870,7 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>200</v>
+        <v>43</v>
       </c>
     </row>
     <row r="24">
@@ -877,7 +885,7 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>1500</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25">
@@ -893,7 +901,7 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2023-01-01 → 2024-12-30</t>
+          <t>2023-02-02 → 2024-12-21</t>
         </is>
       </c>
     </row>
@@ -910,7 +918,7 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03 05:36:08</t>
+          <t>2026-08-05 01:34:27</t>
         </is>
       </c>
     </row>
@@ -929,7 +937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -959,245 +967,235 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-02</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>129535.27</v>
+        <v>1544.25</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>124177.15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2023-04</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>94687.5</v>
+        <v>4767.04</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2023-05</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>120211.39</v>
+        <v>1396.05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-06</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>214979.4</v>
+        <v>1244.76</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2023-07</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>144172.33</v>
+        <v>2068.36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>79795.75999999999</v>
+        <v>1192.18</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>95892.77</v>
+        <v>2459.11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>131471.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>130650.4</v>
+        <v>3098.64</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>134301.94</v>
+        <v>2538.74</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>98102.98</v>
+        <v>2115.88</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>100712.49</v>
+        <v>708.36</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>95156.14999999999</v>
+        <v>1643.64</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>152135.03</v>
+        <v>1358.05</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>179150.19</v>
+        <v>1085.52</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>93727.07000000001</v>
+        <v>2695.74</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>136878.22</v>
+        <v>4228.88</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>144719.91</v>
+        <v>880.98</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>82512.99000000001</v>
+        <v>2122.44</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>111494.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>105083.01</v>
+        <v>6283.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>186283.31</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>144684.09</v>
+        <v>2962.83</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:B27"/>
+  <autoFilter ref="A3:B26"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
@@ -1245,7 +1243,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>348399.92</v>
+        <v>1544.25</v>
       </c>
     </row>
     <row r="5">
@@ -1255,7 +1253,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>479363.12</v>
+        <v>7407.85</v>
       </c>
     </row>
     <row r="6">
@@ -1265,7 +1263,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>307160.15</v>
+        <v>5719.65</v>
       </c>
     </row>
     <row r="7">
@@ -1275,7 +1273,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>363055.32</v>
+        <v>5637.38</v>
       </c>
     </row>
     <row r="8">
@@ -1285,7 +1283,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>348003.67</v>
+        <v>4467.88</v>
       </c>
     </row>
     <row r="9">
@@ -1295,7 +1293,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>409755.48</v>
+        <v>5139.31</v>
       </c>
     </row>
     <row r="10">
@@ -1305,7 +1303,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>338727.13</v>
+        <v>7232.3</v>
       </c>
     </row>
     <row r="11">
@@ -1315,7 +1313,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>436050.41</v>
+        <v>9246.530000000001</v>
       </c>
     </row>
   </sheetData>
@@ -1333,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1375,85 +1373,21 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>CRM Enterprise</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>1803012.32</v>
+        <v>46395.15</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>59.5</v>
+        <v>100</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>CRM Pro</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>634008.13</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>20.92</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>CRM Basic</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>220106.44</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>7.26</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Training</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>216364.72</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>7.14</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>554</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Support Pack</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>157023.59</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>581</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D8"/>
+  <autoFilter ref="A3:D4"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -1467,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1513,81 +1447,17 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>790180.45</v>
+        <v>46395.15</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>230</v>
+        <v>40</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>3435.57</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Istanbul</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>606547.28</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>188</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>3226.32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Izmir</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>602272.99</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>163</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>3694.93</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Antalya</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>554342.78</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>159</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>3486.43</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Ankara</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>477171.7</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>149</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>3202.49</v>
+        <v>1159.88</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:D8"/>
+  <autoFilter ref="A3:D4"/>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
@@ -1635,7 +1505,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>889</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -1645,7 +1515,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>291</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -1655,7 +1525,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>320</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -1665,7 +1535,7 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>75.34</v>
+        <v>68.97</v>
       </c>
     </row>
     <row r="8">
@@ -1675,7 +1545,7 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>21.33</v>
+        <v>18.31</v>
       </c>
     </row>
     <row r="9">
@@ -1686,7 +1556,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>AM_5</t>
+          <t>AM_1</t>
         </is>
       </c>
     </row>
@@ -1697,7 +1567,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>678845.98</v>
+        <v>14930.24</v>
       </c>
     </row>
   </sheetData>
@@ -1731,7 +1601,7 @@
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1821,44 +1691,44 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>258</v>
+        <v>13</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>153</v>
+        <v>8</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>585640.4300000001</v>
+        <v>10632.1</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>19.32</v>
+        <v>22.92</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>15411.59</v>
+        <v>1518.87</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>3827.72</v>
+        <v>1329.01</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>76.5</v>
+        <v>72.73</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>22.48</v>
+        <v>15.38</v>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>CRM Enterprise</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
@@ -1869,44 +1739,44 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>101</v>
+        <v>17</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>757</v>
+        <v>25</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>456</v>
+        <v>14</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>142</v>
+        <v>5</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>159</v>
+        <v>6</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>1477615.56</v>
+        <v>14895.2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>48.76</v>
+        <v>32.11</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>14629.86</v>
+        <v>876.1900000000001</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>3240.38</v>
+        <v>1063.94</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>76.25</v>
+        <v>73.68000000000001</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>CRM Enterprise</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
@@ -1917,44 +1787,44 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>485</v>
+        <v>33</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>280</v>
+        <v>18</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>967259.21</v>
+        <v>20867.85</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>31.92</v>
+        <v>44.98</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>15856.71</v>
+        <v>1098.31</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>3454.5</v>
+        <v>1159.32</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>73.3</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>21.24</v>
+        <v>15.15</v>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>CRM Enterprise</t>
+          <t>Training</t>
         </is>
       </c>
     </row>
@@ -2015,415 +1885,409 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-01</t>
+          <t>2023-02</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>129535.27</v>
+        <v>1544.25</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>122987.17</v>
+        <v>1439.76</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2023-02</t>
+          <t>2023-03</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>124177.15</v>
+        <v>0</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>123272.76</v>
+        <v>1492.25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2023-03</t>
+          <t>2023-04</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>94687.5</v>
+        <v>4767.04</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>123558.35</v>
+        <v>1544.74</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2023-04</t>
+          <t>2023-05</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>120211.39</v>
+        <v>1396.05</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>123843.95</v>
+        <v>1597.24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2023-05</t>
+          <t>2023-06</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>214979.4</v>
+        <v>1244.76</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>124129.54</v>
+        <v>1649.73</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2023-06</t>
+          <t>2023-07</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>144172.33</v>
+        <v>2068.36</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>124415.13</v>
+        <v>1702.22</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2023-07</t>
+          <t>2023-08</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>79795.75999999999</v>
+        <v>1192.18</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>124700.72</v>
+        <v>1754.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2023-08</t>
+          <t>2023-09</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>95892.77</v>
+        <v>2459.11</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>124986.31</v>
+        <v>1807.21</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2023-09</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>131471.62</v>
+        <v>0</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>125271.9</v>
+        <v>1859.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2023-11</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>130650.4</v>
+        <v>3098.64</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>125557.49</v>
+        <v>1912.19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2023-11</t>
+          <t>2023-12</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>134301.94</v>
+        <v>2538.74</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>125843.08</v>
+        <v>1964.69</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2023-12</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>98102.98</v>
+        <v>2115.88</v>
       </c>
       <c r="C15" s="9" t="n">
-        <v>126128.67</v>
+        <v>2017.18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>100712.49</v>
+        <v>708.36</v>
       </c>
       <c r="C16" s="9" t="n">
-        <v>126414.26</v>
+        <v>2069.67</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-03</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>95156.14999999999</v>
+        <v>1643.64</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>126699.85</v>
+        <v>2122.17</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2024-03</t>
+          <t>2024-04</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>152135.03</v>
+        <v>1358.05</v>
       </c>
       <c r="C18" s="9" t="n">
-        <v>126985.44</v>
+        <v>2174.66</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2024-04</t>
+          <t>2024-05</t>
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>179150.19</v>
+        <v>1085.52</v>
       </c>
       <c r="C19" s="9" t="n">
-        <v>127271.03</v>
+        <v>2227.15</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2024-05</t>
+          <t>2024-06</t>
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>93727.07000000001</v>
+        <v>2695.74</v>
       </c>
       <c r="C20" s="9" t="n">
-        <v>127556.62</v>
+        <v>2279.65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2024-06</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>136878.22</v>
+        <v>4228.88</v>
       </c>
       <c r="C21" s="9" t="n">
-        <v>127842.22</v>
+        <v>2332.14</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-08</t>
         </is>
       </c>
       <c r="B22" s="9" t="n">
-        <v>144719.91</v>
+        <v>880.98</v>
       </c>
       <c r="C22" s="9" t="n">
-        <v>128127.81</v>
+        <v>2384.63</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2024-08</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>82512.99000000001</v>
+        <v>2122.44</v>
       </c>
       <c r="C23" s="9" t="n">
-        <v>128413.4</v>
+        <v>2437.13</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>111494.23</v>
+        <v>0</v>
       </c>
       <c r="C24" s="9" t="n">
-        <v>128698.99</v>
+        <v>2489.62</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>105083.01</v>
+        <v>6283.7</v>
       </c>
       <c r="C25" s="9" t="n">
-        <v>128984.58</v>
+        <v>2542.11</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>186283.31</v>
+        <v>2962.83</v>
       </c>
       <c r="C26" s="9" t="n">
-        <v>129270.17</v>
+        <v>2594.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="n">
-        <v>144684.09</v>
-      </c>
-      <c r="C27" s="9" t="n">
-        <v>129555.76</v>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="n">
+        <v>2647.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="D28" s="9" t="n">
-        <v>129841.35</v>
+        <v>2699.59</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="D29" s="9" t="n">
-        <v>130126.94</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2025-03</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="n">
-        <v>130412.53</v>
-      </c>
-    </row>
+        <v>2752.08</v>
+      </c>
+    </row>
+    <row r="30"/>
     <row r="31"/>
-    <row r="32"/>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Linear Regression</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Method</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Linear Regression</t>
+          <t>NumPy polyfit</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>NumPy polyfit</t>
-        </is>
+          <t>Slope</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>52.49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Slope</t>
+          <t>R²</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>285.59</v>
+        <v>0.0534</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R²</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>0.0036</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
           <t>Trend Direction</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
-      </c>
-    </row>
-    <row r="38"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Growing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Forecast Assumptions</t>
+        </is>
+      </c>
+    </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Forecast Assumptions</t>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>The forecast is based only on historical monthly revenue.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>The forecast is based only on historical monthly revenue.</t>
+          <t>Missing calendar months are retained with zero revenue.</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2409,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Month-over-month revenue changed by -22.33%.</t>
+          <t>Month-over-month revenue changed by -52.85%.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -2580,7 +2444,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>21.33% of order records have the 'Churned' status.</t>
+          <t>18.31% of order records have the 'Churned' status.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -2596,31 +2460,31 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Warning</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Overall revenue trend is stable</t>
+          <t>Revenue concentrated in one product</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Linear trend slope is 285.59 per month and remains within the stability tolerance.</t>
+          <t>'Training' contributes 100.0% of total revenue.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Monitor upcoming periods and focus on converting stable performance into sustainable growth.</t>
+          <t>Increase cross-selling and upselling of other products to reduce concentration risk.</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2497,7 @@
       <c r="B7" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -2650,7 +2514,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Bursa generated the highest revenue at 790,180.45. Izmir had the highest average order value at 3,694.93.</t>
+          <t>Bursa generated the highest revenue at 46,395.15. Bursa had the highest average order value at 1,159.88.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2668,7 +2532,7 @@
       <c r="B8" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
@@ -2685,7 +2549,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Win rate is 75.34%.</t>
+          <t>Win rate is 68.97%.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -2703,29 +2567,29 @@
       <c r="B9" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Product revenue reasonably diversified</t>
+          <t>Overall revenue trend is growing</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>The largest product share is 59.5% from 'CRM Enterprise'.</t>
+          <t>Linear trend slope is 52.49 per month.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Maintain product diversification while monitoring changes in revenue concentration.</t>
+          <t>Use the current trend as a reference when setting future sales targets.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2619,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Aylık gelir değişimi -22.33% olarak gerçekleşti.</t>
+          <t>Aylık gelir değişimi -52.85% olarak gerçekleşti.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -2790,7 +2654,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Sipariş kayıtlarının %21.33 kadarı 'Churned' durumundadır.</t>
+          <t>Sipariş kayıtlarının %18.31 kadarı 'Churned' durumundadır.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -2806,31 +2670,31 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Warning</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Ürün</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Genel gelir trendi sabit</t>
+          <t>Gelir tek bir üründe yoğunlaşmış</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Doğrusal trend eğimi aylık 285.59 seviyesindedir ve kararlılık toleransı içinde kalmaktadır.</t>
+          <t>'Training' toplam gelirin %100.0 kadarını oluşturmaktadır.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Gelecek dönemleri takip edin ve sabit performansı sürdürülebilir büyümeye dönüştürmeye odaklanın.</t>
+          <t>Yoğunlaşma riskini azaltmak için diğer ürünlerde çapraz satış ve üst satış çalışmalarını artırın.</t>
         </is>
       </c>
     </row>
@@ -2843,7 +2707,7 @@
       <c r="B13" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -2860,7 +2724,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Bursa, 790,180.45 ile en yüksek geliri elde etti. Izmir, 3,694.93 ile en yüksek ortalama sipariş değerine ulaştı.</t>
+          <t>Bursa, 46,395.15 ile en yüksek geliri elde etti. Bursa, 1,159.88 ile en yüksek ortalama sipariş değerine ulaştı.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -2878,7 +2742,7 @@
       <c r="B14" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
@@ -2895,7 +2759,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Kazanma oranı %75.34.</t>
+          <t>Kazanma oranı %68.97.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -2913,29 +2777,29 @@
       <c r="B15" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Ürün</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Ürün gelir dağılımı yeterince çeşitlendirilmiş</t>
+          <t>Genel gelir trendi yükseliyor</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>En büyük ürün payı, 'CRM Enterprise' ürünüyle %59.5 seviyesindedir.</t>
+          <t>Doğrusal trend eğimi aylık 52.49 seviyesindedir.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Gelir yoğunluğundaki değişimleri takip ederken ürün çeşitliliğini koruyun.</t>
+          <t>Gelecekteki satış hedeflerini belirlerken mevcut trendi referans olarak kullanın.</t>
         </is>
       </c>
     </row>

</xml_diff>